<commit_message>
feat: add initial UI implementation and update README
</commit_message>
<xml_diff>
--- a/data/results/[20250831] IQT-1 Checkride 1/20250831_landing_results.xlsx
+++ b/data/results/[20250831] IQT-1 Checkride 1/20250831_landing_results.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,35 +512,25 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>td_longitude</t>
+          <t>CAS_kt</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>td_latitude</t>
+          <t>VS_fpm</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>CAS_kt</t>
+          <t>Airport</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>VS_fpm</t>
+          <t>Runway</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
-        <is>
-          <t>Airport</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Runway</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
         <is>
           <t>touchdown_to_threshold_ft</t>
         </is>
@@ -567,28 +557,22 @@
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>145.7264342</v>
+        <v>173</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>15.1177538</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>173</v>
-      </c>
-      <c r="I2" s="3" t="n">
         <v>-501</v>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Saipan</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>07R</t>
         </is>
       </c>
-      <c r="L2" s="3" t="n">
+      <c r="J2" s="3" t="n">
         <v>3127</v>
       </c>
     </row>
@@ -613,28 +597,22 @@
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>144.9246307</v>
+        <v>172</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>13.5843089</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>172</v>
-      </c>
-      <c r="I3" s="6" t="n">
         <v>-69</v>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Andersen</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>06L</t>
         </is>
       </c>
-      <c r="L3" s="6" t="n">
+      <c r="J3" s="6" t="n">
         <v>3427</v>
       </c>
     </row>
@@ -659,28 +637,22 @@
         </is>
       </c>
       <c r="F4" s="8" t="n">
-        <v>144.9191412</v>
+        <v>173</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>13.5821251</v>
-      </c>
-      <c r="H4" s="8" t="n">
-        <v>173</v>
-      </c>
-      <c r="I4" s="8" t="n">
         <v>-198</v>
       </c>
-      <c r="J4" s="8" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>Andersen</t>
         </is>
       </c>
-      <c r="K4" s="8" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>06L</t>
         </is>
       </c>
-      <c r="L4" s="8" t="n">
+      <c r="J4" s="8" t="n">
         <v>1327</v>
       </c>
     </row>
@@ -705,28 +677,22 @@
         </is>
       </c>
       <c r="F5" s="12" t="n">
-        <v>144.9171175</v>
+        <v>162</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>13.5809588</v>
-      </c>
-      <c r="H5" s="12" t="n">
-        <v>162</v>
-      </c>
-      <c r="I5" s="12" t="n">
         <v>-190</v>
       </c>
-      <c r="J5" s="12" t="inlineStr">
+      <c r="H5" s="12" t="inlineStr">
         <is>
           <t>Andersen</t>
         </is>
       </c>
-      <c r="K5" s="12" t="inlineStr">
+      <c r="I5" s="12" t="inlineStr">
         <is>
           <t>06L</t>
         </is>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="J5" s="12" t="n">
         <v>496</v>
       </c>
     </row>
@@ -751,28 +717,22 @@
         </is>
       </c>
       <c r="F6" s="14" t="n">
-        <v>144.9209473</v>
+        <v>157</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>13.5826299</v>
-      </c>
-      <c r="H6" s="14" t="n">
-        <v>157</v>
-      </c>
-      <c r="I6" s="14" t="n">
         <v>-387</v>
       </c>
-      <c r="J6" s="14" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>Andersen</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
+      <c r="I6" s="14" t="inlineStr">
         <is>
           <t>06L</t>
         </is>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="J6" s="14" t="n">
         <v>1985</v>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: migrate to vectorized csv runway database
</commit_message>
<xml_diff>
--- a/data/results/[20250831] IQT-1 Checkride 1/20250831_landing_results.xlsx
+++ b/data/results/[20250831] IQT-1 Checkride 1/20250831_landing_results.xlsx
@@ -564,16 +564,16 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Saipan</t>
+          <t>PGSN</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>07R</t>
+          <t>07</t>
         </is>
       </c>
       <c r="J2" s="3" t="n">
-        <v>3127</v>
+        <v>3198</v>
       </c>
     </row>
     <row r="3">
@@ -604,7 +604,7 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Andersen</t>
+          <t>PGUA</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="J3" s="6" t="n">
-        <v>3427</v>
+        <v>3391</v>
       </c>
     </row>
     <row r="4">
@@ -644,7 +644,7 @@
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>Andersen</t>
+          <t>PGUA</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="J4" s="8" t="n">
-        <v>1327</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="5">
@@ -684,7 +684,7 @@
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>Andersen</t>
+          <t>PGUA</t>
         </is>
       </c>
       <c r="I5" s="12" t="inlineStr">
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
-        <v>496</v>
+        <v>463</v>
       </c>
     </row>
     <row r="6">
@@ -724,7 +724,7 @@
       </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>Andersen</t>
+          <t>PGUA</t>
         </is>
       </c>
       <c r="I6" s="14" t="inlineStr">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>1985</v>
+        <v>1949</v>
       </c>
     </row>
   </sheetData>

</xml_diff>